<commit_message>
UK rental: integrate 2024 data from spreadsheet, update tax-year totals
</commit_message>
<xml_diff>
--- a/projects/uk-rental/mortgage-monthly.xlsx
+++ b/projects/uk-rental/mortgage-monthly.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Monthly mortgage" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tax summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,19 +418,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,27 +446,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Opening (£)</t>
+          <t>Opening (GBP)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Interest charged (£)</t>
+          <t>Interest charged (GBP)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Capital paid (£)</t>
+          <t>Capital paid (GBP)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Product fee (£)</t>
+          <t>Product fee (GBP)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Closing (£)</t>
+          <t>Closing (GBP)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -968,7 +967,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -976,39 +975,39 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>178999.86</v>
+        <v>189805.22</v>
       </c>
       <c r="D14" t="n">
-        <v>222.26</v>
+        <v>234.52</v>
       </c>
       <c r="E14" t="n">
-        <v>718.0700000000001</v>
+        <v>1405.82</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>178281.79</v>
+        <v>188399.4</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1016,39 +1015,39 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>178281.79</v>
+        <v>188171.42</v>
       </c>
       <c r="D15" t="n">
-        <v>221.37</v>
+        <v>232.81</v>
       </c>
       <c r="E15" t="n">
-        <v>718.95</v>
+        <v>1407.57</v>
       </c>
       <c r="F15" t="n">
-        <v>1749</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>179311.84</v>
+        <v>186763.85</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1056,39 +1055,39 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>179311.84</v>
+        <v>186763.89</v>
       </c>
       <c r="D16" t="n">
-        <v>638.98</v>
+        <v>231.9</v>
       </c>
       <c r="E16" t="n">
-        <v>546.9</v>
+        <v>1408.48</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>178764.94</v>
+        <v>185355.41</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1096,39 +1095,39 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>178764.94</v>
+        <v>185354.58</v>
       </c>
       <c r="D17" t="n">
-        <v>652.49</v>
+        <v>458.55</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>2822.21</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>178764.94</v>
+        <v>182532.37</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024 (2 rows)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1136,39 +1135,39 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>178764.94</v>
+        <v>182530.71</v>
       </c>
       <c r="D18" t="n">
-        <v>652.49</v>
+        <v>451.53</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>2829.23</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>178764.94</v>
+        <v>179701.48</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024 (2 rows)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1176,39 +1175,39 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>178764.94</v>
+        <v>179699.87</v>
       </c>
       <c r="D19" t="n">
-        <v>652.49</v>
+        <v>444.5</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1436.21</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>178764.94</v>
+        <v>178263.66</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024 (2 rows)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1216,39 +1215,39 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>178764.94</v>
+        <v>177565.43</v>
       </c>
       <c r="D20" t="n">
-        <v>652.49</v>
+        <v>2397.11</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>546.9</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>178764.94</v>
+        <v>177018.53</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024 - anomalous</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1262,27 +1261,27 @@
         <v>652.49</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>-0.49</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>178764.94</v>
+        <v>178765.43</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>spreadsheet 2024 - projection?</t>
         </is>
       </c>
     </row>
@@ -1292,27 +1291,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>178764.94</v>
+        <v>178999.86</v>
       </c>
       <c r="D22" t="n">
-        <v>652.49</v>
+        <v>222.26</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>718.0700000000001</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>178764.94</v>
+        <v>178281.79</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1332,27 +1331,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>178764.94</v>
+        <v>178281.79</v>
       </c>
       <c r="D23" t="n">
-        <v>652.49</v>
+        <v>221.37</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>718.95</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1749</v>
       </c>
       <c r="G23" t="n">
-        <v>178764.94</v>
+        <v>179311.84</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1372,17 +1371,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>178764.94</v>
+        <v>179311.84</v>
       </c>
       <c r="D24" t="n">
-        <v>652.49</v>
+        <v>638.98</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>546.9</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
@@ -1392,7 +1391,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1412,7 +1411,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1432,7 +1431,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1448,11 +1447,11 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>May</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1477,22 +1476,22 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1517,22 +1516,22 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1557,22 +1556,22 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1597,22 +1596,22 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1632,15 +1631,335 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2025 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D31" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2025 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D32" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2025 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D33" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2025 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D34" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D35" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D36" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D37" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D38" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>26/27</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>2026 PDF</t>
         </is>
@@ -1657,14 +1976,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1682,17 +2002,22 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Mortgage interest (£)</t>
+          <t>Interest (GBP)</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Product fees (£)</t>
+          <t>Fees (GBP)</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Total deductible (£)</t>
+          <t>Total (GBP)</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Coverage</t>
         </is>
       </c>
     </row>
@@ -1711,6 +2036,11 @@
       <c r="D3" t="n">
         <v>1023.29</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Partial - Jan-Mar 2023 only</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1719,13 +2049,18 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1989.77</v>
+        <v>3147.55</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>1989.77</v>
+        <v>3147.55</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Partial - Apr-Dec 2023 + Jan-Mar 2024 (2024 data from spreadsheet)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1735,13 +2070,18 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1735.1</v>
+        <v>5680.73</v>
       </c>
       <c r="C5" t="n">
         <v>1749</v>
       </c>
       <c r="D5" t="n">
-        <v>3484.1</v>
+        <v>7429.73</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Apr 2024-Mar 2025 (2024 from spreadsheet w/ caveats)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1759,6 +2099,11 @@
       <c r="D6" t="n">
         <v>7829.88</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Full year (statement)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1775,6 +2120,11 @@
       <c r="D7" t="n">
         <v>652.49</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Partial - May 2026 only</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1791,17 +2141,22 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Mortgage interest (£)</t>
+          <t>Interest (GBP)</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Product fees (£)</t>
+          <t>Fees (GBP)</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>Total deductible (£)</t>
+          <t>Total (GBP)</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Coverage</t>
         </is>
       </c>
     </row>
@@ -1820,191 +2175,72 @@
       <c r="D11" t="n">
         <v>3013.06</v>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Full year (statement)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6955.02</v>
+        <v>5103.41</v>
       </c>
       <c r="C12" t="n">
-        <v>1749</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>8704.02</v>
+        <v>5103.41</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Partial - Jan-Aug from spreadsheet only, Sep-Dec MISSING</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3262.45</v>
+        <v>6955.02</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1749</v>
       </c>
       <c r="D13" t="n">
-        <v>3262.45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>76a Ingelow Road — Santander mortgage monthly tracker</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Account: 0915/862/044470945/MOR | Started: 21 Jan 2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MORTGAGE PRODUCT HISTORY</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>21 Jan 2020 → 02 Feb 2025: 1.49% fixed, REPAYMENT, monthly £940.33</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>03 Feb 2025 → 02 May 2027: 4.38% fixed, INTEREST ONLY, monthly £652.49 (product fee £1,749)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ERC if paid off before 02/05/2027: £3,575.30</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>DATA SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2023: 2023 annual statement PDF (full year)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2024: NOT IN PROVIDED PDFs — request 2024 annual statement to fill gap</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2025: 2025 annual statement PDF (full year)</t>
+        <v>8704.02</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Full year (statement)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026 Jan-May: Online banking PDF (interest-only continuation)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>UNRESOLVED: ~£234.92 balance discrepancy</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Spreadsheet's last 'actual closing' (Aug 2024) was £178,764.94.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Statement's 1 Jan 2025 opening is £178,999.86 — up £234.92.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>During 2025 the balance net DECREASED by £234.92 (back to £178,764.94).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>The two figures match exactly — likely the same fee/adjustment booked in late 2024 and reversed in 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Hypothesis: a small interim charge near the product switch (Feb 2025) was held in late 2024 and netted out in 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Cannot confirm without 2024 annual statement.</t>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3262.45</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3262.45</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Partial - Jan-May only</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UK rental: derive 2024 cleanly from rate+DD+overpay; reconciles to Jan 2025 within £0.08
</commit_message>
<xml_diff>
--- a/projects/uk-rental/mortgage-monthly.xlsx
+++ b/projects/uk-rental/mortgage-monthly.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -430,7 +430,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -975,19 +975,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>189805.22</v>
+        <v>195880.1</v>
       </c>
       <c r="D14" t="n">
-        <v>234.52</v>
+        <v>243.22</v>
       </c>
       <c r="E14" t="n">
-        <v>1405.82</v>
+        <v>1397.11</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>188399.4</v>
+        <v>194482.99</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>spreadsheet 2024</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1015,19 +1015,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>188171.42</v>
+        <v>194482.99</v>
       </c>
       <c r="D15" t="n">
-        <v>232.81</v>
+        <v>241.48</v>
       </c>
       <c r="E15" t="n">
-        <v>1407.57</v>
+        <v>1398.85</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>186763.85</v>
+        <v>193084.14</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>spreadsheet 2024</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1055,19 +1055,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>186763.89</v>
+        <v>193084.14</v>
       </c>
       <c r="D16" t="n">
-        <v>231.9</v>
+        <v>239.75</v>
       </c>
       <c r="E16" t="n">
-        <v>1408.48</v>
+        <v>1400.58</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>185355.41</v>
+        <v>191683.56</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>spreadsheet 2024</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1095,19 +1095,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>185354.58</v>
+        <v>191683.56</v>
       </c>
       <c r="D17" t="n">
-        <v>458.55</v>
+        <v>238.01</v>
       </c>
       <c r="E17" t="n">
-        <v>2822.21</v>
+        <v>1402.32</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>182532.37</v>
+        <v>190281.24</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>spreadsheet 2024 (2 rows)</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1135,19 +1135,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>182530.71</v>
+        <v>190281.24</v>
       </c>
       <c r="D18" t="n">
-        <v>451.53</v>
+        <v>236.27</v>
       </c>
       <c r="E18" t="n">
-        <v>2829.23</v>
+        <v>1404.06</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>179701.48</v>
+        <v>188877.18</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>spreadsheet 2024 (2 rows)</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1175,19 +1175,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>179699.87</v>
+        <v>188877.18</v>
       </c>
       <c r="D19" t="n">
-        <v>444.5</v>
+        <v>234.52</v>
       </c>
       <c r="E19" t="n">
-        <v>1436.21</v>
+        <v>1405.81</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>178263.66</v>
+        <v>187471.37</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>spreadsheet 2024 (2 rows)</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1215,19 +1215,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>177565.43</v>
+        <v>187471.37</v>
       </c>
       <c r="D20" t="n">
-        <v>2397.11</v>
+        <v>232.78</v>
       </c>
       <c r="E20" t="n">
-        <v>546.9</v>
+        <v>1407.55</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>177018.53</v>
+        <v>186063.82</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>spreadsheet 2024 - anomalous</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1255,19 +1255,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>178764.94</v>
+        <v>186063.82</v>
       </c>
       <c r="D21" t="n">
-        <v>652.49</v>
+        <v>231.03</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.49</v>
+        <v>1409.3</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>178765.43</v>
+        <v>184654.52</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1281,33 +1281,33 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>spreadsheet 2024 - projection?</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>178999.86</v>
+        <v>184654.52</v>
       </c>
       <c r="D22" t="n">
-        <v>222.26</v>
+        <v>229.28</v>
       </c>
       <c r="E22" t="n">
-        <v>718.0700000000001</v>
+        <v>1411.05</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>178281.79</v>
+        <v>183243.47</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1316,38 +1316,38 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>178281.79</v>
+        <v>183243.47</v>
       </c>
       <c r="D23" t="n">
-        <v>221.37</v>
+        <v>227.53</v>
       </c>
       <c r="E23" t="n">
-        <v>718.95</v>
+        <v>1412.8</v>
       </c>
       <c r="F23" t="n">
-        <v>1749</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>179311.84</v>
+        <v>181830.67</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1356,38 +1356,38 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Nov</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>179311.84</v>
+        <v>181830.67</v>
       </c>
       <c r="D24" t="n">
-        <v>638.98</v>
+        <v>225.77</v>
       </c>
       <c r="E24" t="n">
-        <v>546.9</v>
+        <v>1414.56</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>178764.94</v>
+        <v>180416.11</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1396,38 +1396,38 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>178764.94</v>
+        <v>180416.11</v>
       </c>
       <c r="D25" t="n">
-        <v>652.49</v>
+        <v>224.02</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1416.31</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>178764.94</v>
+        <v>178999.8</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1436,12 +1436,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2025 PDF</t>
+          <t>derived (1.49% + DD £940.33 + overpay £700)</t>
         </is>
       </c>
     </row>
@@ -1451,27 +1451,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>178764.94</v>
+        <v>178999.86</v>
       </c>
       <c r="D26" t="n">
-        <v>652.49</v>
+        <v>222.26</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>718.0700000000001</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>178764.94</v>
+        <v>178281.79</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1491,27 +1491,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>178764.94</v>
+        <v>178281.79</v>
       </c>
       <c r="D27" t="n">
-        <v>652.49</v>
+        <v>221.37</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>718.95</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1749</v>
       </c>
       <c r="G27" t="n">
-        <v>178764.94</v>
+        <v>179311.84</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1531,17 +1531,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jul</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>178764.94</v>
+        <v>179311.84</v>
       </c>
       <c r="D28" t="n">
-        <v>652.49</v>
+        <v>638.98</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>546.9</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>May</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nov</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1767,11 +1767,11 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1796,22 +1796,22 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Feb</t>
+          <t>Oct</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1836,22 +1836,22 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Nov</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1876,22 +1876,22 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Dec</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1916,12 +1916,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026 PDF</t>
+          <t>2025 PDF</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1931,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1951,15 +1951,175 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D39" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D40" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D41" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026 PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="D42" t="n">
+        <v>652.49</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>178764.94</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
           <t>26/27</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>2026 PDF</t>
         </is>
@@ -2049,17 +2209,17 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3147.55</v>
+        <v>2952.23</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>3147.55</v>
+        <v>2952.23</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Partial - Apr-Dec 2023 + Jan-Mar 2024 (2024 data from spreadsheet)</t>
+          <t>Full year (Apr-Dec 2023 PDF + Jan-Mar 2024 derived)</t>
         </is>
       </c>
     </row>
@@ -2070,17 +2230,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5680.73</v>
+        <v>3576.3</v>
       </c>
       <c r="C5" t="n">
         <v>1749</v>
       </c>
       <c r="D5" t="n">
-        <v>7429.73</v>
+        <v>5325.3</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Apr 2024-Mar 2025 (2024 from spreadsheet w/ caveats)</t>
+          <t>Full year (Apr-Dec 2024 derived + Jan-Mar 2025 PDF)</t>
         </is>
       </c>
     </row>
@@ -2188,17 +2348,17 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5103.41</v>
+        <v>2803.66</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>5103.41</v>
+        <v>2803.66</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Partial - Jan-Aug from spreadsheet only, Sep-Dec MISSING</t>
+          <t>Full year (derived; reconciles to Jan 2025 statement open within £0.08)</t>
         </is>
       </c>
     </row>

</xml_diff>